<commit_message>
Update ENSEMBLE pipeline outputs and docs
</commit_message>
<xml_diff>
--- a/studySpecific/ENSEMBLE/テスト実施記録_CombineProcess.xlsx
+++ b/studySpecific/ENSEMBLE/テスト実施記録_CombineProcess.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Local\iTMS\SDTM_ENSEMBLE\studySpecific\ENSEMBLE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2EF9CD7-5DF4-4FE8-BCD9-60A96241A0CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E103048-63C2-401D-AE3F-DD7BA2023803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="727" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="727" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="表紙" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="105">
   <si>
     <t>VC_BC05_studyFunctions モジュール</t>
   </si>
@@ -74,9 +74,6 @@
   </si>
   <si>
     <t>レビュー者</t>
-  </si>
-  <si>
-    <t>Group B</t>
   </si>
   <si>
     <t>承認者</t>
@@ -180,9 +177,6 @@
     <t>Git Commit</t>
   </si>
   <si>
-    <t>WIP</t>
-  </si>
-  <si>
     <t>テスト実施記録</t>
     <phoneticPr fontId="6"/>
   </si>
@@ -365,6 +359,10 @@
   </si>
   <si>
     <t>張　泊江（Group A）</t>
+  </si>
+  <si>
+    <t>96985d9</t>
+    <phoneticPr fontId="6"/>
   </si>
 </sst>
 </file>
@@ -921,7 +919,7 @@
   <sheetData>
     <row r="2" spans="2:3" ht="28.5" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="2:3" ht="18.75" x14ac:dyDescent="0.2">
@@ -942,7 +940,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.15">
@@ -950,7 +948,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.15">
@@ -974,34 +972,32 @@
         <v>4</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.15">
       <c r="B13" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.15">
       <c r="B14" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="14" t="s">
-        <v>16</v>
-      </c>
+      <c r="C14" s="14"/>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.15">
       <c r="B15" s="14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C15" s="14"/>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.15">
       <c r="B16" s="14" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C16" s="14" t="s">
         <v>2</v>
@@ -1009,10 +1005,10 @@
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.15">
       <c r="B17" s="14" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1033,7 +1029,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="17.25" x14ac:dyDescent="0.15">
       <c r="A1" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="12" customFormat="1" x14ac:dyDescent="0.15">
@@ -1041,23 +1037,23 @@
         <v>12</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A4" s="16" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" s="16" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.15">
@@ -1065,23 +1061,23 @@
         <v>5</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A7" s="16" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A8" s="16" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1107,272 +1103,272 @@
   <sheetData>
     <row r="1" spans="1:8" ht="17.25" x14ac:dyDescent="0.15">
       <c r="A1" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>20</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>24</v>
-      </c>
       <c r="G4" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H4" s="14"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>27</v>
-      </c>
       <c r="G5" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H5" s="14"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>30</v>
-      </c>
       <c r="G6" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H6" s="14"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>32</v>
-      </c>
       <c r="G7" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H7" s="14"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A8" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>35</v>
-      </c>
       <c r="G8" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H8" s="14"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A9" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" s="14" t="s">
-        <v>38</v>
-      </c>
       <c r="G9" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H9" s="14"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="C10" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>41</v>
-      </c>
       <c r="G10" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H10" s="14"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A11" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="C11" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>44</v>
-      </c>
       <c r="G11" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H11" s="14"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A12" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="D12" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C12" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="F12" s="14" t="s">
-        <v>97</v>
-      </c>
       <c r="G12" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H12" s="14"/>
     </row>
     <row r="13" spans="1:8" ht="27" x14ac:dyDescent="0.15">
       <c r="A13" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="C13" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="D13" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="C13" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="E13" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" s="22" t="s">
-        <v>101</v>
-      </c>
       <c r="G13" s="21" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H13" s="21"/>
     </row>
@@ -1397,7 +1393,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17.25" x14ac:dyDescent="0.15">
       <c r="A1" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17.25" x14ac:dyDescent="0.15">
@@ -1405,33 +1401,33 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A3" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="D3" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="E3" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="F3" s="8" t="s">
         <v>79</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A4" s="6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>11</v>
@@ -1440,7 +1436,7 @@
         <v>11</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1464,22 +1460,22 @@
   <sheetData>
     <row r="1" spans="1:1" ht="17.25" x14ac:dyDescent="0.15">
       <c r="A1" s="10" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A3" s="20" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A4" s="20" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A5" s="20" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1499,29 +1495,29 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.25" x14ac:dyDescent="0.15">
       <c r="A1" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A3" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>91</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>93</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A4" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -1539,7 +1535,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A6" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -1567,7 +1563,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.25" x14ac:dyDescent="0.15">
       <c r="A1" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.15">
@@ -1584,24 +1580,24 @@
         <v>10</v>
       </c>
       <c r="E3" s="24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A4" s="25" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B4" s="26">
         <v>46073</v>
       </c>
       <c r="C4" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="E4" s="28" t="s">
         <v>104</v>
-      </c>
-      <c r="D4" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="E4" s="28" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>